<commit_message>
publica clinica-sorriso-valparaiso top-odonto-valparaiso vivaz-odontologia oral-vita-radiologia instituto-neves
</commit_message>
<xml_diff>
--- a/follow_up.xlsx
+++ b/follow_up.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -508,7 +508,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>enviado</t>
+          <t>dormante</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -518,20 +518,20 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2a tentativa (saida digna) em 2026-07-23</t>
+          <t>reabertura so com gatilho novo (30+ dias)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>ciclo1 - 1o toque enviado 18/07 | 2o toque reagendado p/ 23/07 (espacamento de 5 dias apos 1o toque)</t>
+          <t>ciclo1 - 1o toque enviado 18/07 | saida digna enviada 25/07 - dormante</t>
         </is>
       </c>
     </row>
@@ -553,7 +553,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>enviado</t>
+          <t>dormante</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -563,20 +563,20 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2a tentativa (saida digna) em 2026-07-23</t>
+          <t>reabertura so com gatilho novo (30+ dias)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>ciclo1 - 1o toque enviado 18/07 | 2o toque reagendado p/ 23/07 (espacamento de 5 dias apos 1o toque)</t>
+          <t>ciclo1 - 1o toque enviado 18/07 | saida digna enviada 25/07 - dormante</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>enviado</t>
+          <t>dormante</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -608,20 +608,20 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2a tentativa (saida digna) em 2026-07-23</t>
+          <t>reabertura so com gatilho novo (30+ dias)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>ciclo1 - 1o toque enviado 18/07 | 2o toque reagendado p/ 23/07 (espacamento de 5 dias apos 1o toque)</t>
+          <t>ciclo1 - 1o toque enviado 18/07 | saida digna enviada 25/07 - dormante</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>enviado</t>
+          <t>dormante</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -653,20 +653,20 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2a tentativa (saida digna) em 2026-07-23</t>
+          <t>reabertura so com gatilho novo (30+ dias)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>ciclo2 - 1o toque enviado 18/07 | 2o toque reagendado p/ 23/07 (espacamento de 5 dias apos 1o toque)</t>
+          <t>ciclo2 - 1o toque enviado 18/07 | saida digna enviada 25/07 - dormante</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>enviado</t>
+          <t>dormante</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -698,20 +698,20 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2a tentativa (saida digna) em 2026-07-23</t>
+          <t>reabertura so com gatilho novo (30+ dias)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>ciclo2 - 1o toque enviado 18/07 | 2o toque reagendado p/ 23/07 (espacamento de 5 dias apos 1o toque)</t>
+          <t>ciclo2 - 1o toque enviado 18/07 | saida digna enviada 25/07 - dormante</t>
         </is>
       </c>
     </row>
@@ -733,7 +733,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>enviado</t>
+          <t>dormante</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -743,20 +743,20 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2a tentativa (saida digna) em 2026-07-23</t>
+          <t>reabertura so com gatilho novo (30+ dias)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>ciclo2 - 1o toque enviado 18/07 | 2o toque reagendado p/ 23/07 (espacamento de 5 dias apos 1o toque)</t>
+          <t>ciclo2 - 1o toque enviado 18/07 | saida digna enviada 25/07 - dormante</t>
         </is>
       </c>
     </row>
@@ -802,6 +802,121 @@
       <c r="J8" t="inlineStr">
         <is>
           <t>respondeu e conversou, mas nao avancou - fora da cadencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>oral-clinica</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Oral Clínica</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>(61) 3060-5029</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>enviado</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>1a tentativa (toque leve) em 2026-07-27</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>ciclo3 - proposta enviada 24/07</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>odontoclin-especialidades</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Odontoclin Especialidades</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>(61) 99947-3584</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>canal_invalido</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>tentar Instagram @odontoclinespecialidades</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>ciclo3 - wa.me do proprio site nao existe como conta</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>mec-odontologia</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MEC Clínica Odontológica</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>(61) 99675-1678</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>enviado</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>1a tentativa (toque leve) em 2026-07-27</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>ciclo3 - proposta enviada 24/07</t>
         </is>
       </c>
     </row>

</xml_diff>